<commit_message>
devel: forms in forms
</commit_message>
<xml_diff>
--- a/configs/schemas/main.xlsx
+++ b/configs/schemas/main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madeliri/Documents/git/shiny_form/configs/schemas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07037598-774F-A843-9C67-26D8CBECEED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D369536-C475-6640-BC0E-BCF413CBA54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="19000" xr2:uid="{9A1397C5-2914-6B46-9457-B60C998D9C07}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="80">
   <si>
     <t>part</t>
   </si>
@@ -264,6 +264,18 @@
   </si>
   <si>
     <t>но значение должно быть между 0 и 250</t>
+  </si>
+  <si>
+    <t>inline_table2</t>
+  </si>
+  <si>
+    <t>example_inline_table_2</t>
+  </si>
+  <si>
+    <t>test_inline2.xlsx</t>
+  </si>
+  <si>
+    <t>Пример вложенной таблицы2</t>
   </si>
 </sst>
 </file>
@@ -714,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DDED1F0-0BDB-364F-8AF4-EDF00BBB7CEB}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="7" customWidth="1"/>
@@ -952,111 +964,119 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="7" t="s">
+      <c r="C16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B17" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C17" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F17" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G17" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="5" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C18" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F19" s="12"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C20" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E20" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
       <c r="F20" s="12"/>
       <c r="G20" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C21" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="H21" s="6"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F22" s="12"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F22" s="12"/>
-      <c r="G22" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
       <c r="F23" s="12"/>
       <c r="G23" s="5" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -1064,104 +1084,109 @@
       <c r="D24" s="6"/>
       <c r="F24" s="12"/>
       <c r="G24" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C25" s="6" t="s">
+      <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C26" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="12"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>67</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>16</v>
       </c>
       <c r="E26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F26" s="12"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B27" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="F26" s="12"/>
-      <c r="H26" s="6"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C27" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="F27" s="12"/>
       <c r="H27" s="6"/>
-      <c r="I27">
-        <v>1</v>
-      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C28" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" t="s">
-        <v>8</v>
+        <v>66</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>7</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>19</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="F28" s="12"/>
       <c r="H28" s="6"/>
       <c r="I28">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A29" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>4</v>
+      <c r="C29" s="6" t="s">
+        <v>63</v>
       </c>
       <c r="D29" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H29" s="6"/>
       <c r="I29">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="F30" s="12"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="1"/>
+      <c r="I30">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F31" s="12"/>
@@ -1185,13 +1210,16 @@
       <c r="F37" s="12"/>
     </row>
     <row r="38" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F38" s="6"/>
+      <c r="F38" s="12"/>
     </row>
     <row r="39" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F39" s="6"/>
     </row>
+    <row r="40" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F40" s="6"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C30:D1048576 C1:C29">
+  <conditionalFormatting sqref="C31:D1048576 C1:C30">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>